<commit_message>
chore(data-release): publish site data 2026-08-10 00:56:50 UTC
</commit_message>
<xml_diff>
--- a/diseases/d003/2000-2004.xlsx
+++ b/diseases/d003/2000-2004.xlsx
@@ -439,110 +439,255 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>record_kind</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>country_code</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>country_name</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>disease_id</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>disease_name_en</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>disease_name_zh</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>year_month</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>cases</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>weekly_equiv_cases</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>deaths</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>incidence_rate_per_100k</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>incidence_rate_source</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>mortality_rate</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>series_code</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>source_series_code</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>source_system</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>source_label</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>metric_type</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>reporting_basis</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>temporal_granularity</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>geography_key</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>dimension_key</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>mapping_relation</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>comparability</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>aggregation_policy</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>availability_status</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>missing_value_policy</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>definition_version</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>case_definition</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>case_definition_uri</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>quality_status</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>is_selected_series</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>data_layer</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>projection_policy</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>coverage_status</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>loss_risk</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>selected_series_codes</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>available_series_count</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>provenance_note</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
         <is>
           <t>primary_source_scope</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>primary_source_label</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>primary_source_url</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>primary_source_type</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>source_scopes</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>source_labels</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>source_urls</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>source_types</t>
         </is>
@@ -571,97 +716,126 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Taiwan, China</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>2003-02-01</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>2003-02</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="n">
-        <v>0.25</v>
-      </c>
       <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
         <v>0.004412259560257887</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="BB2" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="BC2" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -690,97 +864,126 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2003-03-01</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>2003-03</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>610</v>
       </c>
-      <c r="N3" t="n">
-        <v>137.7419354838709</v>
-      </c>
       <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
+        <v>610</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
         <v>8.893545931847882</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="AW3" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="AX3" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="BA3" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="BB3" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="BC3" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -809,97 +1012,126 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Taiwan, China</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2003-03-01</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>2003-03</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>14</v>
       </c>
-      <c r="N4" t="n">
-        <v>3.5</v>
-      </c>
       <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
         <v>0.06177163384361041</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="AW4" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="AX4" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="BA4" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="BB4" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="BC4" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -928,97 +1160,126 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2003-04-01</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>2003-04</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>979</v>
       </c>
-      <c r="N5" t="n">
-        <v>221.0645161290323</v>
-      </c>
       <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
+        <v>979</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
         <v>14.27341224144111</v>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="AW5" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="AX5" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="BA5" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="BB5" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="BC5" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1047,97 +1308,126 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Taiwan, China</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2003-04-01</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>2003-04</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>197</v>
       </c>
-      <c r="N6" t="n">
-        <v>44.48387096774194</v>
-      </c>
       <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
+        <v>197</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
         <v>0.8692151333708037</v>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="AW6" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="AX6" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="BA6" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="BB6" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="BC6" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1166,97 +1456,126 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2003-05-01</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>2003-05</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>150</v>
       </c>
-      <c r="N7" t="n">
-        <v>35</v>
-      </c>
       <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
+        <v>150</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
         <v>2.186937524224889</v>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="AW7" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="AX7" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="BA7" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="BB7" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="BC7" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1285,97 +1604,126 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Taiwan, China</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2003-05-01</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>2003-05</t>
         </is>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>238</v>
       </c>
-      <c r="N8" t="n">
-        <v>55.53333333333333</v>
-      </c>
       <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
+        <v>238</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
         <v>1.050117775341377</v>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="AW8" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="AX8" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="BA8" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="BB8" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="BC8" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1404,97 +1752,126 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2003-06-01</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>2003-06</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>16</v>
       </c>
-      <c r="N9" t="n">
-        <v>3.612903225806452</v>
-      </c>
       <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
         <v>0.2332733359173215</v>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="AW9" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="AX9" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="BA9" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="BB9" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="BC9" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1523,97 +1900,126 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Taiwan, China</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2003-06-01</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>2003-06</t>
         </is>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>14</v>
       </c>
-      <c r="N10" t="n">
-        <v>3.161290322580645</v>
-      </c>
       <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
         <v>0.06177163384361041</v>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="AW10" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="AX10" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="BA10" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="BB10" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="BC10" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1642,97 +2048,126 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2003-07-01</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>2003-07</t>
         </is>
       </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="AW11" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="AX11" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="BA11" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="BB11" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="BC11" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1761,97 +2196,126 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2003-08-01</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>2003-08</t>
         </is>
       </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
       <c r="N12" t="n">
         <v>0</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="AW12" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="AX12" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W12" t="inlineStr">
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="BA12" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="BB12" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="BC12" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1880,97 +2344,126 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>2003-09-01</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>2003-09</t>
         </is>
       </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="inlineStr">
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="AW13" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="AX13" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="BA13" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="BB13" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="BC13" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -1999,97 +2492,126 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>2003-10-01</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>2003-10</t>
         </is>
       </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="inlineStr">
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="AW14" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="AX14" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="BA14" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="BB14" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="BC14" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2118,97 +2640,126 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>2003-11-01</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>2003-11</t>
         </is>
       </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="inlineStr">
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="AW15" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="AX15" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="BA15" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="BB15" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="BC15" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2237,97 +2788,126 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>2003-12-01</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>2003-12</t>
         </is>
       </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
       <c r="N16" t="n">
         <v>0</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="inlineStr">
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="AW16" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="AX16" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="BA16" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="BB16" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr">
+      <c r="BC16" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2356,97 +2936,126 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Taiwan, China</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>2003-12-01</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>2003-12</t>
         </is>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>1</v>
       </c>
-      <c r="N17" t="n">
-        <v>0.03825136612021858</v>
-      </c>
       <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
         <v>0.004412259560257887</v>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="AW17" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="AX17" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
         <is>
           <t>nidss_open_data</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="BA17" t="inlineStr">
         <is>
           <t>Taiwan, China CDC NIDSS</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="BB17" t="inlineStr">
         <is>
           <t>https://nidss.cdc.gov.tw/Home/Index</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="BC17" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2475,97 +3084,126 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>2004-01-01</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>2004-01</t>
         </is>
       </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
       <c r="N18" t="n">
         <v>0</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="inlineStr">
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="AW18" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="AX18" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
+      <c r="BA18" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="BB18" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="BC18" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2594,97 +3232,126 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>2004-02-01</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>2004-02</t>
         </is>
       </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="inlineStr">
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="AW19" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="AX19" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="BA19" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="BB19" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="BC19" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2713,97 +3380,126 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>2004-03-01</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>2004-03</t>
         </is>
       </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
       <c r="N20" t="n">
         <v>0</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="inlineStr">
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="AW20" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="AX20" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W20" t="inlineStr">
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="BA20" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="BB20" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="BC20" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2832,97 +3528,126 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>2004-04-01</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>2004-04</t>
         </is>
       </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
       <c r="N21" t="n">
         <v>0</v>
       </c>
       <c r="O21" t="n">
         <v>0</v>
       </c>
-      <c r="P21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="inlineStr">
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="AW21" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="AX21" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr">
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="BA21" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="BB21" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="BC21" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -2951,97 +3676,126 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>2004-05-01</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>2004-05</t>
         </is>
       </c>
-      <c r="M22" t="n">
-        <v>0</v>
-      </c>
       <c r="N22" t="n">
         <v>0</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
       </c>
-      <c r="P22" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" t="inlineStr">
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="AW22" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="AX22" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W22" t="inlineStr">
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ22" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="BA22" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
+      <c r="BB22" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="BC22" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3070,97 +3824,126 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>2004-06-01</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>2004-06</t>
         </is>
       </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
       <c r="N23" t="n">
         <v>0</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="inlineStr">
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="AW23" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="AX23" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ23" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="BA23" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
+      <c r="BB23" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="BC23" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3189,97 +3972,126 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>2004-07-01</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>2004-07</t>
         </is>
       </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
       <c r="N24" t="n">
         <v>0</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="inlineStr">
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV24" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="AW24" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="AX24" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W24" t="inlineStr">
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ24" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="BA24" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="BB24" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="BC24" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3308,97 +4120,126 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>2004-08-01</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>2004-08</t>
         </is>
       </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
       <c r="N25" t="n">
         <v>0</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
-      <c r="P25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="inlineStr">
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="AW25" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="AX25" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr">
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ25" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="BA25" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="BB25" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="BC25" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3427,97 +4268,126 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>2004-09-01</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>2004-09</t>
         </is>
       </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
-      <c r="P26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV26" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="AW26" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="AX26" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ26" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="BA26" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
+      <c r="BB26" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z26" t="inlineStr">
+      <c r="BC26" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3546,97 +4416,126 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>2004-10-01</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>2004-10</t>
         </is>
       </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV27" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="AW27" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="AX27" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
+      <c r="AY27" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ27" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="BA27" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
+      <c r="BB27" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z27" t="inlineStr">
+      <c r="BC27" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3665,97 +4564,126 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>2004-11-01</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>2004-11</t>
         </is>
       </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="inlineStr">
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV28" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="AW28" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="AX28" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
+      <c r="AY28" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ28" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
+      <c r="BA28" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
+      <c r="BB28" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z28" t="inlineStr">
+      <c r="BC28" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3784,97 +4712,126 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>HK</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Hong Kong, China</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>D003</t>
-        </is>
-      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>SARS</t>
+          <t>D003</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>SARS</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
           <t>传染性非典型肺炎</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>2004-12-01</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>2004-12</t>
         </is>
       </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="inlineStr">
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP29" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV29" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="AW29" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="AX29" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>open_data_csv</t>
-        </is>
-      </c>
-      <c r="W29" t="inlineStr">
+      <c r="AY29" t="inlineStr">
+        <is>
+          <t>open_data_csv</t>
+        </is>
+      </c>
+      <c r="AZ29" t="inlineStr">
         <is>
           <t>chp_notifiable</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="BA29" t="inlineStr">
         <is>
           <t>Hong Kong, China CHP Notifiable Diseases</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
+      <c r="BB29" t="inlineStr">
         <is>
           <t>https://www.chp.gov.hk/en/static/24012.html</t>
         </is>
       </c>
-      <c r="Z29" t="inlineStr">
+      <c r="BC29" t="inlineStr">
         <is>
           <t>open_data_csv</t>
         </is>
@@ -3992,7 +4949,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>record_count</t>
+          <t>projection_record_count</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4002,27 +4959,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>schema_version</t>
+          <t>record_count</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>total_cases</t>
+          <t>schema_version</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2220</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>total_deaths</t>
+          <t>source_observation_count</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4032,22 +4989,64 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>window_end</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2004-12-31</t>
-        </is>
+          <t>source_series_count</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>total_basis</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>total_cases</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>total_deaths</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>window_end</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2004-12-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>window_start</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>2000-01-01</t>
         </is>

</xml_diff>